<commit_message>
Corrections, événements, arrêts de produit et substitutions, version arbitrée (modèle v0.9)
Nouvel onglet Corrections (saisie, annulation), calcul de la quantité retenue dans PREVISION,
colonne Qte substitution, écran Prévision détaillé. 109 tests.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VDUD2te9mLDL4jRRkQGkWq
</commit_message>
<xml_diff>
--- a/modeles/xlsx/SORTIE_SOP.xlsx
+++ b/modeles/xlsx/SORTIE_SOP.xlsx
@@ -93,7 +93,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modèle de structure v0.8 – à compléter. L'application contrôle que les onglets et colonnes correspondent à cette version.</t>
+          <t xml:space="preserve">Modèle de structure v0.9 – à compléter. L'application contrôle que les onglets et colonnes correspondent à cette version.</t>
         </is>
       </c>
     </row>
@@ -1197,6 +1197,7 @@
     <col min="18" max="18" width="24" customWidth="1"/>
     <col min="19" max="19" width="15" customWidth="1"/>
     <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1298,6 +1299,11 @@
       <c r="T1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Modifie le</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Qte substitution</t>
         </is>
       </c>
     </row>

</xml_diff>